<commit_message>
Apply client changes: Persian digits, result caption, scheduler, updated images and excel
</commit_message>
<xml_diff>
--- a/Quizbot/data/RESULT_IMAGES.xlsx
+++ b/Quizbot/data/RESULT_IMAGES.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\++My Codes\Web Develop\Telegam_Bale Bot\Keramat_Quizbot2\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\++My Codes\Web Develop\Telegam_Bale Bot\Keramat_Quizbot2\Quizbot\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11D76329-F3B4-4DF2-AF9F-6E89F4D8B02E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF5FEEC1-5C76-44D3-8937-C14C77FCFE2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,19 +33,19 @@
     <t>image</t>
   </si>
   <si>
-    <t>Borj.jpg</t>
-  </si>
-  <si>
-    <t>Bagh.jpg</t>
-  </si>
-  <si>
-    <t>Durbin.jpg</t>
-  </si>
-  <si>
-    <t>pardaz.jpg</t>
-  </si>
-  <si>
-    <t>damp.jpg</t>
+    <t>Borj.png</t>
+  </si>
+  <si>
+    <t>Bagh.png</t>
+  </si>
+  <si>
+    <t>Durbin.png</t>
+  </si>
+  <si>
+    <t>pardaz.png</t>
+  </si>
+  <si>
+    <t>damp.png</t>
   </si>
 </sst>
 </file>

</xml_diff>